<commit_message>
fix: enforce exactly 400 test cases in E2E and Security reports
</commit_message>
<xml_diff>
--- a/backend/Security_Vulnerability_Report_2026-06-11T07-29-57.xlsx
+++ b/backend/Security_Vulnerability_Report_2026-06-11T07-29-57.xlsx
@@ -18386,7 +18386,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -18403,7 +18403,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -18420,7 +18420,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -18437,7 +18437,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -18454,7 +18454,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -18471,7 +18471,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -18488,7 +18488,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -18505,7 +18505,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -18522,7 +18522,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -18539,7 +18539,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -18556,7 +18556,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -18573,7 +18573,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -18590,7 +18590,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -18607,7 +18607,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -18624,7 +18624,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -18641,7 +18641,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -18658,7 +18658,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -18675,7 +18675,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -18692,7 +18692,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -18709,7 +18709,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -18726,7 +18726,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -18743,7 +18743,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -18760,7 +18760,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -18777,7 +18777,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -18794,7 +18794,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -18811,7 +18811,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -18828,7 +18828,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -18845,7 +18845,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -18862,7 +18862,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -18879,7 +18879,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -18896,7 +18896,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -18913,7 +18913,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -18930,7 +18930,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -18947,7 +18947,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -18964,7 +18964,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -18981,7 +18981,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -18998,7 +18998,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -19015,7 +19015,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -19032,7 +19032,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -19049,7 +19049,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -19066,7 +19066,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -19083,7 +19083,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -19100,7 +19100,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -19117,7 +19117,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -19134,7 +19134,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -19151,7 +19151,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -19168,7 +19168,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -19185,7 +19185,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -19202,7 +19202,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -19219,7 +19219,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -19236,7 +19236,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -19253,7 +19253,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -19270,7 +19270,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -19287,7 +19287,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -19304,7 +19304,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -19321,7 +19321,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -19338,7 +19338,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -19355,7 +19355,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -19372,7 +19372,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -19389,7 +19389,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -19406,7 +19406,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -19423,7 +19423,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -19440,7 +19440,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -19457,7 +19457,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -19474,7 +19474,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -19491,7 +19491,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -19508,7 +19508,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -19525,7 +19525,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -19542,7 +19542,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -19559,7 +19559,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -19576,7 +19576,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -19593,7 +19593,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -19610,7 +19610,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -19627,7 +19627,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -19644,7 +19644,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -19661,7 +19661,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -19678,7 +19678,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -19695,7 +19695,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -19712,7 +19712,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -19729,7 +19729,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -19746,7 +19746,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -19763,7 +19763,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -19780,7 +19780,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -19797,7 +19797,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -19814,7 +19814,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -19831,7 +19831,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -19848,7 +19848,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -19865,7 +19865,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -19882,7 +19882,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -19899,7 +19899,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -19916,7 +19916,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -19933,7 +19933,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -19950,7 +19950,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -19967,7 +19967,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -19984,7 +19984,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -20001,7 +20001,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -20018,7 +20018,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -20035,7 +20035,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -20052,7 +20052,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -20069,7 +20069,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -20086,7 +20086,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -20103,7 +20103,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -20120,7 +20120,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -20137,7 +20137,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -20154,7 +20154,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -20171,7 +20171,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -20188,7 +20188,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -20205,7 +20205,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -20222,7 +20222,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -20239,7 +20239,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -20256,7 +20256,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -20273,7 +20273,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -20290,7 +20290,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -20307,7 +20307,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -20324,7 +20324,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -20341,7 +20341,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -20358,7 +20358,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -20375,7 +20375,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -20392,7 +20392,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -20409,7 +20409,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -20426,7 +20426,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -20443,7 +20443,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -20460,7 +20460,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -20477,7 +20477,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -20494,7 +20494,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -20511,7 +20511,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -20528,7 +20528,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -20545,7 +20545,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -20562,7 +20562,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -20579,7 +20579,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -20596,7 +20596,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -20613,7 +20613,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -20630,7 +20630,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -20647,7 +20647,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -20664,7 +20664,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -20681,7 +20681,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -20698,7 +20698,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -20715,7 +20715,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -20732,7 +20732,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -20749,7 +20749,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -20766,7 +20766,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -20783,7 +20783,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -20800,7 +20800,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -20817,7 +20817,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -20834,7 +20834,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -20851,7 +20851,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -20868,7 +20868,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -20885,7 +20885,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -20902,7 +20902,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -20919,7 +20919,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -20936,7 +20936,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -20953,7 +20953,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -20970,7 +20970,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -20987,7 +20987,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
@@ -21004,7 +21004,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -21021,7 +21021,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -21038,7 +21038,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -21055,7 +21055,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -21072,7 +21072,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
@@ -21089,7 +21089,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -21106,7 +21106,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -21123,7 +21123,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -21140,7 +21140,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -21157,7 +21157,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -21174,7 +21174,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -21191,7 +21191,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -21208,7 +21208,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -21225,7 +21225,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -21242,7 +21242,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -21259,7 +21259,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -21276,7 +21276,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -21293,7 +21293,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -21310,7 +21310,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -21327,7 +21327,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -21344,7 +21344,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -21361,7 +21361,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -21378,7 +21378,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -21395,7 +21395,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -21412,7 +21412,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -21429,7 +21429,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -21446,7 +21446,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -21463,7 +21463,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -21480,7 +21480,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -21497,7 +21497,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -21514,7 +21514,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -21531,7 +21531,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -21548,7 +21548,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -21565,7 +21565,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -21582,7 +21582,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -21599,7 +21599,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -21616,7 +21616,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -21633,7 +21633,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -21650,7 +21650,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -21667,7 +21667,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -21684,7 +21684,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -21701,7 +21701,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -21718,7 +21718,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -21735,7 +21735,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -21752,7 +21752,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -21769,7 +21769,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -21786,7 +21786,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -21803,7 +21803,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -21820,7 +21820,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -21837,7 +21837,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -21854,7 +21854,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -21871,7 +21871,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -21888,7 +21888,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -21905,7 +21905,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -21922,7 +21922,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -21939,7 +21939,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -21956,7 +21956,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -21973,7 +21973,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -21990,7 +21990,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -22007,7 +22007,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
@@ -22024,7 +22024,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
@@ -22041,7 +22041,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -22058,7 +22058,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -22075,7 +22075,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
@@ -22092,7 +22092,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
@@ -22109,7 +22109,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
@@ -22126,7 +22126,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -22143,7 +22143,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -22160,7 +22160,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -22177,7 +22177,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -22194,7 +22194,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -22211,7 +22211,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
@@ -22228,7 +22228,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
@@ -22245,7 +22245,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
@@ -22262,7 +22262,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -22279,7 +22279,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -22296,7 +22296,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
@@ -22313,7 +22313,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
@@ -22330,7 +22330,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
@@ -22347,7 +22347,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
@@ -22364,7 +22364,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
@@ -22381,7 +22381,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
@@ -22398,7 +22398,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
@@ -22415,7 +22415,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
@@ -22432,7 +22432,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
@@ -22449,7 +22449,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
@@ -22466,7 +22466,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
@@ -22483,7 +22483,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
@@ -22500,7 +22500,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
@@ -22517,7 +22517,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
@@ -22534,7 +22534,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
@@ -22551,7 +22551,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
@@ -22568,7 +22568,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
@@ -22585,7 +22585,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
@@ -22602,7 +22602,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -22619,7 +22619,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
@@ -22636,7 +22636,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
@@ -22653,7 +22653,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
@@ -22670,7 +22670,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
@@ -22687,7 +22687,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
@@ -22704,7 +22704,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
@@ -22721,7 +22721,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
@@ -22738,7 +22738,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
@@ -22755,7 +22755,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
@@ -22772,7 +22772,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
@@ -22789,7 +22789,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
@@ -22806,7 +22806,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
@@ -22823,7 +22823,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
@@ -22840,7 +22840,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
@@ -22857,7 +22857,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
@@ -22874,7 +22874,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
@@ -22891,7 +22891,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
@@ -22908,7 +22908,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
@@ -22925,7 +22925,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
@@ -22942,7 +22942,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
@@ -22959,7 +22959,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -22976,7 +22976,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -22993,7 +22993,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
@@ -23010,7 +23010,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
@@ -23027,7 +23027,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
@@ -23044,7 +23044,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
@@ -23061,7 +23061,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
@@ -23078,7 +23078,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
@@ -23095,7 +23095,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
@@ -23112,7 +23112,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
@@ -23129,7 +23129,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
@@ -23146,7 +23146,7 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
@@ -23163,7 +23163,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
@@ -23180,7 +23180,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
@@ -23197,7 +23197,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
@@ -23214,7 +23214,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
@@ -23231,7 +23231,7 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
@@ -23248,7 +23248,7 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
@@ -23265,7 +23265,7 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
@@ -23282,7 +23282,7 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
@@ -23299,7 +23299,7 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
@@ -23316,7 +23316,7 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
@@ -23333,7 +23333,7 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
@@ -23350,7 +23350,7 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
@@ -23367,7 +23367,7 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
@@ -23384,7 +23384,7 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
@@ -23401,7 +23401,7 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
@@ -23418,7 +23418,7 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
@@ -23435,7 +23435,7 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
@@ -23452,7 +23452,7 @@
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
@@ -23469,7 +23469,7 @@
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
@@ -23486,7 +23486,7 @@
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
@@ -23503,7 +23503,7 @@
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
@@ -23520,7 +23520,7 @@
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
@@ -23537,7 +23537,7 @@
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
@@ -23554,7 +23554,7 @@
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
@@ -23571,7 +23571,7 @@
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
@@ -23588,7 +23588,7 @@
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
@@ -23605,7 +23605,7 @@
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
@@ -23622,7 +23622,7 @@
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
@@ -23639,7 +23639,7 @@
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
@@ -23656,7 +23656,7 @@
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
@@ -23673,7 +23673,7 @@
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
@@ -23690,7 +23690,7 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
@@ -23707,7 +23707,7 @@
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
@@ -23724,7 +23724,7 @@
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
@@ -23741,7 +23741,7 @@
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
@@ -23758,7 +23758,7 @@
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
@@ -23775,7 +23775,7 @@
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
@@ -23792,7 +23792,7 @@
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
@@ -23809,7 +23809,7 @@
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
@@ -23826,7 +23826,7 @@
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
@@ -23843,7 +23843,7 @@
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
@@ -23860,7 +23860,7 @@
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
@@ -23877,7 +23877,7 @@
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
@@ -23894,7 +23894,7 @@
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
@@ -23911,7 +23911,7 @@
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
@@ -23928,7 +23928,7 @@
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
@@ -23945,7 +23945,7 @@
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
@@ -23962,7 +23962,7 @@
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
@@ -23979,7 +23979,7 @@
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
@@ -23996,7 +23996,7 @@
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
@@ -24013,7 +24013,7 @@
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
@@ -24030,7 +24030,7 @@
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
@@ -24047,7 +24047,7 @@
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
@@ -24064,7 +24064,7 @@
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
@@ -24081,7 +24081,7 @@
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
@@ -24098,7 +24098,7 @@
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
@@ -24115,7 +24115,7 @@
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
@@ -24132,7 +24132,7 @@
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
@@ -24149,7 +24149,7 @@
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
@@ -24166,7 +24166,7 @@
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
@@ -24183,7 +24183,7 @@
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
@@ -24200,7 +24200,7 @@
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
@@ -24217,7 +24217,7 @@
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
@@ -24234,7 +24234,7 @@
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B368" t="inlineStr">
@@ -24251,7 +24251,7 @@
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B369" t="inlineStr">
@@ -24268,7 +24268,7 @@
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
@@ -24285,7 +24285,7 @@
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
@@ -24302,7 +24302,7 @@
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B372" t="inlineStr">
@@ -24319,7 +24319,7 @@
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
@@ -24336,7 +24336,7 @@
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B374" t="inlineStr">
@@ -24353,7 +24353,7 @@
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B375" t="inlineStr">
@@ -24370,7 +24370,7 @@
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
@@ -24387,7 +24387,7 @@
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B377" t="inlineStr">
@@ -24404,7 +24404,7 @@
     <row r="378">
       <c r="A378" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B378" t="inlineStr">
@@ -24421,7 +24421,7 @@
     <row r="379">
       <c r="A379" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B379" t="inlineStr">
@@ -24438,7 +24438,7 @@
     <row r="380">
       <c r="A380" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B380" t="inlineStr">
@@ -24455,7 +24455,7 @@
     <row r="381">
       <c r="A381" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B381" t="inlineStr">
@@ -24472,7 +24472,7 @@
     <row r="382">
       <c r="A382" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B382" t="inlineStr">
@@ -24489,7 +24489,7 @@
     <row r="383">
       <c r="A383" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B383" t="inlineStr">
@@ -24506,7 +24506,7 @@
     <row r="384">
       <c r="A384" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B384" t="inlineStr">
@@ -24523,7 +24523,7 @@
     <row r="385">
       <c r="A385" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B385" t="inlineStr">
@@ -24540,7 +24540,7 @@
     <row r="386">
       <c r="A386" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B386" t="inlineStr">
@@ -24557,7 +24557,7 @@
     <row r="387">
       <c r="A387" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B387" t="inlineStr">
@@ -24574,7 +24574,7 @@
     <row r="388">
       <c r="A388" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B388" t="inlineStr">
@@ -24591,7 +24591,7 @@
     <row r="389">
       <c r="A389" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B389" t="inlineStr">
@@ -24608,7 +24608,7 @@
     <row r="390">
       <c r="A390" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B390" t="inlineStr">
@@ -24625,7 +24625,7 @@
     <row r="391">
       <c r="A391" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B391" t="inlineStr">
@@ -24642,7 +24642,7 @@
     <row r="392">
       <c r="A392" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B392" t="inlineStr">
@@ -24659,7 +24659,7 @@
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B393" t="inlineStr">
@@ -24676,7 +24676,7 @@
     <row r="394">
       <c r="A394" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B394" t="inlineStr">
@@ -24693,7 +24693,7 @@
     <row r="395">
       <c r="A395" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B395" t="inlineStr">
@@ -24710,7 +24710,7 @@
     <row r="396">
       <c r="A396" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B396" t="inlineStr">
@@ -24727,7 +24727,7 @@
     <row r="397">
       <c r="A397" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B397" t="inlineStr">
@@ -24744,7 +24744,7 @@
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B398" t="inlineStr">
@@ -24761,7 +24761,7 @@
     <row r="399">
       <c r="A399" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B399" t="inlineStr">
@@ -24778,7 +24778,7 @@
     <row r="400">
       <c r="A400" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B400" t="inlineStr">
@@ -24795,7 +24795,7 @@
     <row r="401">
       <c r="A401" t="inlineStr">
         <is>
-          <t>2026-06-22 18:48:01</t>
+          <t>2026-06-22 19:19:43</t>
         </is>
       </c>
       <c r="B401" t="inlineStr">

</xml_diff>